<commit_message>
Limit mealworm options to 1kg
What changed:

- Generate only small, medium, and large 1kg rows for mealworm SmartStore options.

- Remove disabled mealworm count rows from the committed workbook.

- Update README and option manual copy so mealworm is described as 1kg-only.

- Reword shared package notes from mealworm count wording to generic product quantity wording.

- Ignore temporary files under exports/options while still tracking the SmartStore workbook.

Why:

- Mealworm is sold only as small, medium, and large 1kg options; count-based wording could confuse SmartStore setup.

Verification:

- npm run export:options

- workbook XML check: 25 data rows, 3 mealworm rows, 0 mealworm non-1kg rows, 0 disabled rows

- npm run build

- git diff --check

Known limitations:

- Stock quantities remain blank until inventory values are provided.
</commit_message>
<xml_diff>
--- a/exports/options/mealworm7th_smartstore_options.xlsx
+++ b/exports/options/mealworm7th_smartstore_options.xlsx
@@ -103,11 +103,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>500마리</t>
+          <t>1kg</t>
         </is>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -116,12 +116,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MW-S-500</t>
+          <t>MW-S-1KG</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -133,16 +133,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>중</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1000마리</t>
+          <t>1kg</t>
         </is>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -151,12 +151,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MW-S-1000</t>
+          <t>MW-M-1KG</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -168,16 +168,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>대</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2000마리</t>
+          <t>1kg</t>
         </is>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -186,19 +186,19 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>MW-S-2000</t>
+          <t>MW-L-1KG</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -208,7 +208,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3000마리</t>
+          <t>500마리</t>
         </is>
       </c>
       <c r="D5">
@@ -221,19 +221,19 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MW-S-3000</t>
+          <t>SW-S-500</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -243,11 +243,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5000마리</t>
+          <t>1000마리</t>
         </is>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -256,19 +256,19 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>MW-S-5000</t>
+          <t>SW-S-1000</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -278,11 +278,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1kg</t>
+          <t>2000마리</t>
         </is>
       </c>
       <c r="D7">
-        <v>2000</v>
+        <v>22000</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -291,7 +291,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>MW-S-1KG</t>
+          <t>SW-S-2000</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -303,21 +303,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>중</t>
+          <t>소</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>500마리</t>
+          <t>3000마리</t>
         </is>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -326,33 +326,33 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>MW-M-500</t>
+          <t>SW-S-3000</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>중</t>
+          <t>소</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1000마리</t>
+          <t>5000마리</t>
         </is>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>73000</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -361,33 +361,33 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>MW-M-1000</t>
+          <t>SW-S-5000</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>중</t>
+          <t>소</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2000마리</t>
+          <t>1kg</t>
         </is>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -396,19 +396,19 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>MW-M-2000</t>
+          <t>SW-S-1KG</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -418,7 +418,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3000마리</t>
+          <t>500마리</t>
         </is>
       </c>
       <c r="D11">
@@ -431,19 +431,19 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>MW-M-3000</t>
+          <t>SW-M-500</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -453,11 +453,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>5000마리</t>
+          <t>1000마리</t>
         </is>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -466,19 +466,19 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>MW-M-5000</t>
+          <t>SW-M-1000</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -488,11 +488,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1kg</t>
+          <t>2000마리</t>
         </is>
       </c>
       <c r="D13">
-        <v>2000</v>
+        <v>22000</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -501,7 +501,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>MW-M-1KG</t>
+          <t>SW-M-2000</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -513,21 +513,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>대</t>
+          <t>중</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>500마리</t>
+          <t>3000마리</t>
         </is>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -536,33 +536,33 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MW-L-500</t>
+          <t>SW-M-3000</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>대</t>
+          <t>중</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1000마리</t>
+          <t>5000마리</t>
         </is>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>73000</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -571,33 +571,33 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>MW-L-1000</t>
+          <t>SW-M-5000</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>대</t>
+          <t>중</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2000마리</t>
+          <t>1kg</t>
         </is>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -606,19 +606,19 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>MW-L-2000</t>
+          <t>SW-M-1KG</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3000마리</t>
+          <t>500마리</t>
         </is>
       </c>
       <c r="D17">
@@ -641,19 +641,19 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>MW-L-3000</t>
+          <t>SW-L-500</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -663,11 +663,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5000마리</t>
+          <t>1000마리</t>
         </is>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -676,19 +676,19 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>MW-L-5000</t>
+          <t>SW-L-1000</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>밀웜</t>
+          <t>슈퍼밀웜</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -698,11 +698,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1kg</t>
+          <t>2000마리</t>
         </is>
       </c>
       <c r="D19">
-        <v>2000</v>
+        <v>22000</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>MW-L-1KG</t>
+          <t>SW-L-2000</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -728,16 +728,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>대</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>500마리</t>
+          <t>3000마리</t>
         </is>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -746,7 +746,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SW-S-500</t>
+          <t>SW-L-3000</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -763,16 +763,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>대</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1000마리</t>
+          <t>5000마리</t>
         </is>
       </c>
       <c r="D21">
-        <v>6000</v>
+        <v>73000</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -781,7 +781,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SW-S-1000</t>
+          <t>SW-L-5000</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -798,16 +798,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>대</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2000마리</t>
+          <t>1kg</t>
         </is>
       </c>
       <c r="D22">
-        <v>22000</v>
+        <v>9000</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -816,7 +816,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>SW-S-2000</t>
+          <t>SW-L-1KG</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -828,21 +828,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>슈퍼밀웜</t>
+          <t>건조밀웜</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>0.5kg</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>3000마리</t>
+          <t>단일</t>
         </is>
       </c>
       <c r="D23">
-        <v>35000</v>
+        <v>8000</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SW-S-3000</t>
+          <t>DMW-0_5KG</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -863,21 +863,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>슈퍼밀웜</t>
+          <t>건조밀웜</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>1kg</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>5000마리</t>
+          <t>단일</t>
         </is>
       </c>
       <c r="D24">
-        <v>73000</v>
+        <v>11000</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>SW-S-5000</t>
+          <t>DMW-1KG</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -898,21 +898,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>슈퍼밀웜</t>
+          <t>건조슈퍼밀웜</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>소</t>
+          <t>0.5kg</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1kg</t>
+          <t>단일</t>
         </is>
       </c>
       <c r="D25">
-        <v>9000</v>
+        <v>11000</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>SW-S-1KG</t>
+          <t>DSW-0_5KG</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -933,21 +933,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>슈퍼밀웜</t>
+          <t>건조슈퍼밀웜</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>중</t>
+          <t>1kg</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>500마리</t>
+          <t>단일</t>
         </is>
       </c>
       <c r="D26">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -956,535 +956,10 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SW-M-500</t>
+          <t>DSW-1KG</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1000마리</t>
-        </is>
-      </c>
-      <c r="D27">
-        <v>6000</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>SW-M-1000</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>2000마리</t>
-        </is>
-      </c>
-      <c r="D28">
-        <v>22000</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>SW-M-2000</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>3000마리</t>
-        </is>
-      </c>
-      <c r="D29">
-        <v>35000</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>SW-M-3000</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>5000마리</t>
-        </is>
-      </c>
-      <c r="D30">
-        <v>73000</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>SW-M-5000</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1kg</t>
-        </is>
-      </c>
-      <c r="D31">
-        <v>9000</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>SW-M-1KG</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>대</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>500마리</t>
-        </is>
-      </c>
-      <c r="D32">
-        <v>0</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>SW-L-500</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>대</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1000마리</t>
-        </is>
-      </c>
-      <c r="D33">
-        <v>6000</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>SW-L-1000</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>대</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>2000마리</t>
-        </is>
-      </c>
-      <c r="D34">
-        <v>22000</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>SW-L-2000</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>대</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>3000마리</t>
-        </is>
-      </c>
-      <c r="D35">
-        <v>35000</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>SW-L-3000</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>대</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>5000마리</t>
-        </is>
-      </c>
-      <c r="D36">
-        <v>73000</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>SW-L-5000</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>대</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1kg</t>
-        </is>
-      </c>
-      <c r="D37">
-        <v>9000</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>SW-L-1KG</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>건조밀웜</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>0.5kg</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>단일</t>
-        </is>
-      </c>
-      <c r="D38">
-        <v>8000</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>DMW-0_5KG</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>건조밀웜</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>1kg</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>단일</t>
-        </is>
-      </c>
-      <c r="D39">
-        <v>11000</v>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>DMW-1KG</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>건조슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>0.5kg</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>단일</t>
-        </is>
-      </c>
-      <c r="D40">
-        <v>11000</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>DSW-0_5KG</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>건조슈퍼밀웜</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>1kg</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>단일</t>
-        </is>
-      </c>
-      <c r="D41">
-        <v>18000</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>DSW-1KG</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>